<commit_message>
docs(submission): sync final 00d req mapping and regenerate workbook
</commit_message>
<xml_diff>
--- a/driving-situation-alert/tmp/submission/excel/submission_final_all_in_one.xlsx
+++ b/driving-situation-alert/tmp/submission/excel/submission_final_all_in_one.xlsx
@@ -25210,7 +25210,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -26000,7 +26000,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Req_110, Req_111, Req_125~Req_129</t>
+          <t>Req_052~Req_056</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -26057,7 +26057,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Req_130~Req_139</t>
+          <t>Req_057~Req_066</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -26114,7 +26114,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Req_148~Req_152</t>
+          <t>Req_075~Req_079</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -26171,7 +26171,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Req_153~Req_155</t>
+          <t>Req_080~Req_082</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -27530,11 +27530,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -27912,7 +27912,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>시스템은 현재 경고가 발생한 이유를 운전자가 이해할 수 있게 보여줘야 한다.</t>
+          <t>시스템은 경고 발생 시점에 경고 원인 코드에 대응하는 문구 1종을 표시해야 한다.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -27942,7 +27942,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>시스템은 동일 조건의 경고가 짧은 시간에 반복 표시되어 운전자가 혼란을 느끼지 않도록 해야 한다.</t>
+          <t>시스템은 동일 조건의 경고 재발 시 1000ms 보호구간 내 중복 표시를 억제해야 한다.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -28212,7 +28212,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>구간 전환 시 경고 표시가 갑자기 사라지거나 빠르게 반복 점멸되지 않아야 한다.</t>
+          <t>시스템은 구간 전환 시작 후 150ms 이내 경고 표시를 목표 상태로 안정화하고 비정상 반복 점멸이 없어야 한다.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -28692,7 +28692,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>동일 입력 조건에서 중재 결과가 항상 동일해야 한다.</t>
+          <t>시스템은 동일 입력 조건을 반복 적용했을 때 항상 동일한 최종 중재 결과를 출력해야 한다.</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -28842,7 +28842,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>모든 경고 문구는 운전자가 주행 중 즉시 이해할 수 있는 짧고 일관된 표현으로 제공되어야 한다.</t>
+          <t>시스템은 경고 문구를 사전 정의된 경고 문구 목록에서 선택해 일관된 형식으로 표시해야 한다.</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -29764,7 +29764,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>시스템은 객체 기반 경고의 발생/해제/강등 이벤트를 추적 가능한 형태로 기록해야 한다.</t>
+          <t>시스템은 객체 기반 경고의 발생/해제/강등 이벤트를 이벤트 유형·시각·원인코드와 함께 기록해야 한다.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -29968,7 +29968,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>시스템은 긴급/구간/객체 경보 이벤트를 공통 포맷으로 기록해야 한다.</t>
+          <t>시스템은 긴급/구간/객체 경보 이벤트를 공통 포맷(유형·우선순위·시각)으로 기록해야 한다.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -30002,7 +30002,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>시스템은 최근 경보 이벤트 이력을 운전자가 조회할 수 있도록 제공해야 한다.</t>
+          <t>시스템은 운전자가 경보 이력 조회를 요청하면 최신 순으로 최근 경보 이벤트를 제공해야 한다.</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -30104,7 +30104,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>시스템은 경고 판정에 사용되는 객체/상태 입력의 유효성 및 신뢰도를 점검하고 기준 미만 입력은 경고 판정에서 제외해야 한다.</t>
+          <t>시스템은 유효성 플래그 또는 신뢰도 기준을 통과하지 못한 입력을 경고 판정에서 제외해야 한다.</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -30138,7 +30138,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>시스템은 경고 핵심 입력이 일정 시간 갱신되지 않으면 stale 상태로 판단하고 보수 경고 정책으로 전환해야 한다.</t>
+          <t>시스템은 경고 핵심 입력이 1000ms 이상 갱신되지 않으면 stale 상태로 전환하고 보수 경고 정책을 적용해야 한다.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -30206,7 +30206,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>시스템은 도메인 경계 통신 상태(헬스 메시지 수신 주기/타임아웃/유효 플래그)를 기반으로 경고 출력 채널의 가용성을 판정해야 한다.</t>
+          <t>시스템은 헬스 메시지 수신 주기/타임아웃/유효 플래그 변화를 반영해 100ms 이내 경고 출력 채널 가용성을 갱신 판정해야 한다.</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -30240,7 +30240,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>시스템은 주 출력 채널 장애 시 사용 가능한 대체 채널로 경고를 지속 제공해야 한다.</t>
+          <t>시스템은 주 출력 채널 장애 시 150ms 이내 사용 가능한 대체 채널로 경고 출력을 전환해야 한다.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -30342,7 +30342,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>시스템은 앰비언트와 클러스터 경고가 동일 경고 맥락을 유지하도록 동기 일관성을 관리해야 한다.</t>
+          <t>시스템은 앰비언트와 클러스터 경고가 동일 경고 맥락으로 유지되도록 채널 동기 불일치를 복원해야 한다.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -31126,9 +31126,9 @@
       <c r="H133" s="2" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="inlineStr">
-        <is>
-          <t>기능 요구사항 (Functional) - 77개</t>
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>분류별 상세 ID 목록(기능/비기능/안전/진단)은 내부 matrix로 관리한다.</t>
         </is>
       </c>
       <c r="B134" s="2" t="n"/>
@@ -31150,16 +31150,12 @@
       <c r="H135" s="2" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="3" t="inlineStr">
-        <is>
-          <t>분류</t>
-        </is>
-      </c>
-      <c r="B136" s="3" t="inlineStr">
-        <is>
-          <t>포함 Req. ID</t>
-        </is>
-      </c>
+      <c r="A136" s="1" t="inlineStr">
+        <is>
+          <t>우선순위 요구사항 요약</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="n"/>
       <c r="C136" s="2" t="n"/>
       <c r="D136" s="2" t="n"/>
       <c r="E136" s="2" t="n"/>
@@ -31168,16 +31164,8 @@
       <c r="H136" s="2" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="inlineStr">
-        <is>
-          <t>기본 경고 동작/표시</t>
-        </is>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
-        <is>
-          <t>Req_001, Req_002, Req_003, Req_004, Req_005, Req_007, Req_008, Req_009, Req_010, Req_011, Req_012, Req_013, Req_014, Req_016, Req_017, Req_018, Req_019, Req_020, Req_021, Req_022, Req_024, Req_025</t>
-        </is>
-      </c>
+      <c r="A137" s="2" t="n"/>
+      <c r="B137" s="2" t="n"/>
       <c r="C137" s="2" t="n"/>
       <c r="D137" s="2" t="n"/>
       <c r="E137" s="2" t="n"/>
@@ -31186,18 +31174,26 @@
       <c r="H137" s="2" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>경고 우선순위/중재</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>Req_026, Req_027, Req_028, Req_029, Req_030, Req_032</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="n"/>
-      <c r="D138" s="2" t="n"/>
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>우선순위 등급</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>기준(중요도/긴급도)</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>개수</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>포함 Req. ID</t>
+        </is>
+      </c>
       <c r="E138" s="2" t="n"/>
       <c r="F138" s="2" t="n"/>
       <c r="G138" s="2" t="n"/>
@@ -31206,16 +31202,24 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>차량 기본 기능 연계</t>
+          <t>Critical (P0)</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Req_037, Req_038, Req_039, Req_040, Req_041, Req_042, Req_043, Req_044, Req_045, Req_046, Req_047, Req_048</t>
-        </is>
-      </c>
-      <c r="C139" s="2" t="n"/>
-      <c r="D139" s="2" t="n"/>
+          <t>상/상</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>45개</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Req_001, Req_003, Req_004, Req_007, Req_009, Req_010, Req_011, Req_012, Req_016, Req_017, Req_021, Req_022, Req_023, Req_024, Req_026, Req_027, Req_028, Req_031, Req_032, Req_034, Req_049, Req_050, Req_051, Req_052, Req_053, Req_054, Req_055, Req_056, Req_057, Req_058, Req_059, Req_061, Req_062, Req_064, Req_066, Req_075, Req_076, Req_078, Req_079, Req_086, Req_090, Req_091, Req_092, Req_093, Req_094</t>
+        </is>
+      </c>
       <c r="E139" s="2" t="n"/>
       <c r="F139" s="2" t="n"/>
       <c r="G139" s="2" t="n"/>
@@ -31224,16 +31228,24 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>객체 위험 경고 기능</t>
+          <t>High (P1)</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Req_049, Req_050, Req_051, Req_052, Req_053, Req_054, Req_055, Req_056, Req_057, Req_058, Req_059, Req_060, Req_061, Req_062, Req_064, Req_066</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="n"/>
-      <c r="D140" s="2" t="n"/>
+          <t>상/중</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>30개</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Req_002, Req_005, Req_008, Req_013, Req_014, Req_018, Req_019, Req_020, Req_025, Req_029, Req_030, Req_035, Req_036, Req_037, Req_038, Req_039, Req_040, Req_041, Req_044, Req_046, Req_047, Req_060, Req_063, Req_069, Req_070, Req_082, Req_083, Req_084, Req_085, Req_095</t>
+        </is>
+      </c>
       <c r="E140" s="2" t="n"/>
       <c r="F140" s="2" t="n"/>
       <c r="G140" s="2" t="n"/>
@@ -31242,32 +31254,32 @@
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>운전자 편의/설정 기능</t>
+          <t>Medium (P2)</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Req_067, Req_068, Req_069, Req_070, Req_071, Req_072, Req_073, Req_074</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="n"/>
-      <c r="D141" s="2" t="n"/>
+          <t>중/중</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>20개</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Req_006, Req_015, Req_033, Req_042, Req_043, Req_045, Req_048, Req_065, Req_067, Req_068, Req_071, Req_072, Req_073, Req_074, Req_077, Req_080, Req_081, Req_087, Req_088, Req_089</t>
+        </is>
+      </c>
       <c r="E141" s="2" t="n"/>
       <c r="F141" s="2" t="n"/>
       <c r="G141" s="2" t="n"/>
       <c r="H141" s="2" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>확장 ECU 연계 후보(후속 승격 대상)</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>Req_083, Req_084, Req_085, Req_086, Req_087, Req_088, Req_089, Req_090, Req_091, Req_092, Req_093, Req_094, Req_095</t>
-        </is>
-      </c>
+      <c r="A142" s="2" t="n"/>
+      <c r="B142" s="2" t="n"/>
       <c r="C142" s="2" t="n"/>
       <c r="D142" s="2" t="n"/>
       <c r="E142" s="2" t="n"/>
@@ -31286,7 +31298,11 @@
       <c r="H143" s="2" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n"/>
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t>안전 등급 요약 (HARA 기준)</t>
+        </is>
+      </c>
       <c r="B144" s="2" t="n"/>
       <c r="C144" s="2" t="n"/>
       <c r="D144" s="2" t="n"/>
@@ -31296,11 +31312,7 @@
       <c r="H144" s="2" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="inlineStr">
-        <is>
-          <t>Req_083~Req_095는 제출 시점 기준 확장 후보이며, 구현/검증 증빙 확보 후 활성 요구사항으로 승격한다.</t>
-        </is>
-      </c>
+      <c r="A145" s="2" t="n"/>
       <c r="B145" s="2" t="n"/>
       <c r="C145" s="2" t="n"/>
       <c r="D145" s="2" t="n"/>
@@ -31310,7 +31322,11 @@
       <c r="H145" s="2" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n"/>
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>본 요약의 대표 Req 표기는 01 문서의 현재 번호 체계(오름차순) 기준으로 유지한다.</t>
+        </is>
+      </c>
       <c r="B146" s="2" t="n"/>
       <c r="C146" s="2" t="n"/>
       <c r="D146" s="2" t="n"/>
@@ -31320,11 +31336,7 @@
       <c r="H146" s="2" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="inlineStr">
-        <is>
-          <t>비기능 요구사항 (Non-Functional) - 18개</t>
-        </is>
-      </c>
+      <c r="A147" s="2" t="n"/>
       <c r="B147" s="2" t="n"/>
       <c r="C147" s="2" t="n"/>
       <c r="D147" s="2" t="n"/>
@@ -31334,28 +31346,52 @@
       <c r="H147" s="2" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n"/>
-      <c r="B148" s="2" t="n"/>
-      <c r="C148" s="2" t="n"/>
-      <c r="D148" s="2" t="n"/>
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>안전 등급</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>개수</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>해당 HARA ID</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>관련 Req (대표)</t>
+        </is>
+      </c>
       <c r="E148" s="2" t="n"/>
       <c r="F148" s="2" t="n"/>
       <c r="G148" s="2" t="n"/>
       <c r="H148" s="2" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="3" t="inlineStr">
-        <is>
-          <t>분류</t>
-        </is>
-      </c>
-      <c r="B149" s="3" t="inlineStr">
-        <is>
-          <t>포함 Req. ID</t>
-        </is>
-      </c>
-      <c r="C149" s="2" t="n"/>
-      <c r="D149" s="2" t="n"/>
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>ASIL C (Locked)</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>3개</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>HC-02, HC-03, HC-05</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Req_011~Req_012, Req_021/Req_026~Req_030, Req_052~Req_056</t>
+        </is>
+      </c>
       <c r="E149" s="2" t="n"/>
       <c r="F149" s="2" t="n"/>
       <c r="G149" s="2" t="n"/>
@@ -31364,16 +31400,24 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>성능/반응/안정성</t>
+          <t>ASIL C (Provisional)</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Req_006, Req_015, Req_023, Req_031, Req_033, Req_063, Req_077</t>
-        </is>
-      </c>
-      <c r="C150" s="2" t="n"/>
-      <c r="D150" s="2" t="n"/>
+          <t>2개</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>HC-06, HC-07</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Req_057~Req_066, Req_075~Req_079</t>
+        </is>
+      </c>
       <c r="E150" s="2" t="n"/>
       <c r="F150" s="2" t="n"/>
       <c r="G150" s="2" t="n"/>
@@ -31382,16 +31426,24 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>표현/HMI 품질</t>
+          <t>ASIL B (Locked)</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Req_034, Req_035, Req_036, Req_080, Req_081, Req_082</t>
-        </is>
-      </c>
-      <c r="C151" s="2" t="n"/>
-      <c r="D151" s="2" t="n"/>
+          <t>2개</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>HC-01, HC-04</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Req_010, Req_023/Req_032/Req_033</t>
+        </is>
+      </c>
       <c r="E151" s="2" t="n"/>
       <c r="F151" s="2" t="n"/>
       <c r="G151" s="2" t="n"/>
@@ -31400,16 +31452,24 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>데이터 신뢰성/가용성</t>
+          <t>ASIL B (Provisional)</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Req_075, Req_076, Req_078, Req_079, Req_093</t>
-        </is>
-      </c>
-      <c r="C152" s="2" t="n"/>
-      <c r="D152" s="2" t="n"/>
+          <t>1개</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>HC-08</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Req_080~Req_082</t>
+        </is>
+      </c>
       <c r="E152" s="2" t="n"/>
       <c r="F152" s="2" t="n"/>
       <c r="G152" s="2" t="n"/>
@@ -31436,9 +31496,9 @@
       <c r="H154" s="2" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="inlineStr">
-        <is>
-          <t>안전 요구사항 (Safety) - 40개</t>
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>안전 등급 상세 판정(원인/상황/S-E-C/안전목표)은 governance/00d_HARA_Worksheet.md를 기준으로 관리한다.</t>
         </is>
       </c>
       <c r="B155" s="2" t="n"/>
@@ -31448,602 +31508,6 @@
       <c r="F155" s="2" t="n"/>
       <c r="G155" s="2" t="n"/>
       <c r="H155" s="2" t="n"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="n"/>
-      <c r="B156" s="2" t="n"/>
-      <c r="C156" s="2" t="n"/>
-      <c r="D156" s="2" t="n"/>
-      <c r="E156" s="2" t="n"/>
-      <c r="F156" s="2" t="n"/>
-      <c r="G156" s="2" t="n"/>
-      <c r="H156" s="2" t="n"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="3" t="inlineStr">
-        <is>
-          <t>분류</t>
-        </is>
-      </c>
-      <c r="B157" s="3" t="inlineStr">
-        <is>
-          <t>포함 Req. ID</t>
-        </is>
-      </c>
-      <c r="C157" s="2" t="n"/>
-      <c r="D157" s="2" t="n"/>
-      <c r="E157" s="2" t="n"/>
-      <c r="F157" s="2" t="n"/>
-      <c r="G157" s="2" t="n"/>
-      <c r="H157" s="2" t="n"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="inlineStr">
-        <is>
-          <t>구간/긴급 경고 안전</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>Req_010, Req_011, Req_012, Req_021, Req_023, Req_024, Req_026, Req_027, Req_028, Req_029, Req_030, Req_031, Req_032, Req_033, Req_034</t>
-        </is>
-      </c>
-      <c r="C158" s="2" t="n"/>
-      <c r="D158" s="2" t="n"/>
-      <c r="E158" s="2" t="n"/>
-      <c r="F158" s="2" t="n"/>
-      <c r="G158" s="2" t="n"/>
-      <c r="H158" s="2" t="n"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>감속 보조/도메인 경계 안전</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>Req_049, Req_050, Req_051, Req_052, Req_053, Req_054, Req_055, Req_056</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="n"/>
-      <c r="D159" s="2" t="n"/>
-      <c r="E159" s="2" t="n"/>
-      <c r="F159" s="2" t="n"/>
-      <c r="G159" s="2" t="n"/>
-      <c r="H159" s="2" t="n"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="inlineStr">
-        <is>
-          <t>객체 기반 위험 경고 안전</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>Req_057, Req_058, Req_059, Req_060, Req_061, Req_062, Req_063, Req_064, Req_066</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="n"/>
-      <c r="D160" s="2" t="n"/>
-      <c r="E160" s="2" t="n"/>
-      <c r="F160" s="2" t="n"/>
-      <c r="G160" s="2" t="n"/>
-      <c r="H160" s="2" t="n"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="inlineStr">
-        <is>
-          <t>강건성/채널 안전</t>
-        </is>
-      </c>
-      <c r="B161" s="2" t="inlineStr">
-        <is>
-          <t>Req_075, Req_076, Req_077, Req_078, Req_079, Req_080, Req_081, Req_082</t>
-        </is>
-      </c>
-      <c r="C161" s="2" t="n"/>
-      <c r="D161" s="2" t="n"/>
-      <c r="E161" s="2" t="n"/>
-      <c r="F161" s="2" t="n"/>
-      <c r="G161" s="2" t="n"/>
-      <c r="H161" s="2" t="n"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="2" t="n"/>
-      <c r="B162" s="2" t="n"/>
-      <c r="C162" s="2" t="n"/>
-      <c r="D162" s="2" t="n"/>
-      <c r="E162" s="2" t="n"/>
-      <c r="F162" s="2" t="n"/>
-      <c r="G162" s="2" t="n"/>
-      <c r="H162" s="2" t="n"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="n"/>
-      <c r="B163" s="2" t="n"/>
-      <c r="C163" s="2" t="n"/>
-      <c r="D163" s="2" t="n"/>
-      <c r="E163" s="2" t="n"/>
-      <c r="F163" s="2" t="n"/>
-      <c r="G163" s="2" t="n"/>
-      <c r="H163" s="2" t="n"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="1" t="inlineStr">
-        <is>
-          <t>진단/모니터링 요구사항 (Diagnostic/Observability) - 11개</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="n"/>
-      <c r="C164" s="2" t="n"/>
-      <c r="D164" s="2" t="n"/>
-      <c r="E164" s="2" t="n"/>
-      <c r="F164" s="2" t="n"/>
-      <c r="G164" s="2" t="n"/>
-      <c r="H164" s="2" t="n"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="n"/>
-      <c r="B165" s="2" t="n"/>
-      <c r="C165" s="2" t="n"/>
-      <c r="D165" s="2" t="n"/>
-      <c r="E165" s="2" t="n"/>
-      <c r="F165" s="2" t="n"/>
-      <c r="G165" s="2" t="n"/>
-      <c r="H165" s="2" t="n"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="3" t="inlineStr">
-        <is>
-          <t>분류</t>
-        </is>
-      </c>
-      <c r="B166" s="3" t="inlineStr">
-        <is>
-          <t>포함 Req. ID</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="n"/>
-      <c r="D166" s="2" t="n"/>
-      <c r="E166" s="2" t="n"/>
-      <c r="F166" s="2" t="n"/>
-      <c r="G166" s="2" t="n"/>
-      <c r="H166" s="2" t="n"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>이벤트 기록/조회</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>Req_065, Req_071, Req_072</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="n"/>
-      <c r="D167" s="2" t="n"/>
-      <c r="E167" s="2" t="n"/>
-      <c r="F167" s="2" t="n"/>
-      <c r="G167" s="2" t="n"/>
-      <c r="H167" s="2" t="n"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>입력/채널 헬스 모니터링</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>Req_075, Req_076, Req_078, Req_093</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="n"/>
-      <c r="D168" s="2" t="n"/>
-      <c r="E168" s="2" t="n"/>
-      <c r="F168" s="2" t="n"/>
-      <c r="G168" s="2" t="n"/>
-      <c r="H168" s="2" t="n"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>안전 전이/강등 관측</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>Req_063, Req_064, Req_077, Req_079</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="n"/>
-      <c r="D169" s="2" t="n"/>
-      <c r="E169" s="2" t="n"/>
-      <c r="F169" s="2" t="n"/>
-      <c r="G169" s="2" t="n"/>
-      <c r="H169" s="2" t="n"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="n"/>
-      <c r="B170" s="2" t="n"/>
-      <c r="C170" s="2" t="n"/>
-      <c r="D170" s="2" t="n"/>
-      <c r="E170" s="2" t="n"/>
-      <c r="F170" s="2" t="n"/>
-      <c r="G170" s="2" t="n"/>
-      <c r="H170" s="2" t="n"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="2" t="n"/>
-      <c r="B171" s="2" t="n"/>
-      <c r="C171" s="2" t="n"/>
-      <c r="D171" s="2" t="n"/>
-      <c r="E171" s="2" t="n"/>
-      <c r="F171" s="2" t="n"/>
-      <c r="G171" s="2" t="n"/>
-      <c r="H171" s="2" t="n"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>분류는 관점 기반 요약이며, 동일 요구사항이 기능/안전/비기능/진단에 중복 포함될 수 있다.</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="n"/>
-      <c r="C172" s="2" t="n"/>
-      <c r="D172" s="2" t="n"/>
-      <c r="E172" s="2" t="n"/>
-      <c r="F172" s="2" t="n"/>
-      <c r="G172" s="2" t="n"/>
-      <c r="H172" s="2" t="n"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="2" t="n"/>
-      <c r="B173" s="2" t="n"/>
-      <c r="C173" s="2" t="n"/>
-      <c r="D173" s="2" t="n"/>
-      <c r="E173" s="2" t="n"/>
-      <c r="F173" s="2" t="n"/>
-      <c r="G173" s="2" t="n"/>
-      <c r="H173" s="2" t="n"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="1" t="inlineStr">
-        <is>
-          <t>우선순위 요구사항 요약</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="n"/>
-      <c r="C174" s="2" t="n"/>
-      <c r="D174" s="2" t="n"/>
-      <c r="E174" s="2" t="n"/>
-      <c r="F174" s="2" t="n"/>
-      <c r="G174" s="2" t="n"/>
-      <c r="H174" s="2" t="n"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="2" t="n"/>
-      <c r="B175" s="2" t="n"/>
-      <c r="C175" s="2" t="n"/>
-      <c r="D175" s="2" t="n"/>
-      <c r="E175" s="2" t="n"/>
-      <c r="F175" s="2" t="n"/>
-      <c r="G175" s="2" t="n"/>
-      <c r="H175" s="2" t="n"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="3" t="inlineStr">
-        <is>
-          <t>우선순위 등급</t>
-        </is>
-      </c>
-      <c r="B176" s="3" t="inlineStr">
-        <is>
-          <t>기준(중요도/긴급도)</t>
-        </is>
-      </c>
-      <c r="C176" s="3" t="inlineStr">
-        <is>
-          <t>개수</t>
-        </is>
-      </c>
-      <c r="D176" s="3" t="inlineStr">
-        <is>
-          <t>포함 Req. ID</t>
-        </is>
-      </c>
-      <c r="E176" s="2" t="n"/>
-      <c r="F176" s="2" t="n"/>
-      <c r="G176" s="2" t="n"/>
-      <c r="H176" s="2" t="n"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>Critical (P0)</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>상/상</t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>45개</t>
-        </is>
-      </c>
-      <c r="D177" s="2" t="inlineStr">
-        <is>
-          <t>Req_001, Req_003, Req_004, Req_007, Req_009, Req_010, Req_011, Req_012, Req_016, Req_017, Req_021, Req_022, Req_023, Req_024, Req_026, Req_027, Req_028, Req_031, Req_032, Req_034, Req_049, Req_050, Req_051, Req_052, Req_053, Req_054, Req_055, Req_056, Req_057, Req_058, Req_059, Req_061, Req_062, Req_064, Req_066, Req_075, Req_076, Req_078, Req_079, Req_086, Req_090, Req_091, Req_092, Req_093, Req_094</t>
-        </is>
-      </c>
-      <c r="E177" s="2" t="n"/>
-      <c r="F177" s="2" t="n"/>
-      <c r="G177" s="2" t="n"/>
-      <c r="H177" s="2" t="n"/>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>High (P1)</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>상/중</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>30개</t>
-        </is>
-      </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>Req_002, Req_005, Req_008, Req_013, Req_014, Req_018, Req_019, Req_020, Req_025, Req_029, Req_030, Req_035, Req_036, Req_037, Req_038, Req_039, Req_040, Req_041, Req_044, Req_046, Req_047, Req_060, Req_063, Req_069, Req_070, Req_082, Req_083, Req_084, Req_085, Req_095</t>
-        </is>
-      </c>
-      <c r="E178" s="2" t="n"/>
-      <c r="F178" s="2" t="n"/>
-      <c r="G178" s="2" t="n"/>
-      <c r="H178" s="2" t="n"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>Medium (P2)</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="inlineStr">
-        <is>
-          <t>중/중</t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>20개</t>
-        </is>
-      </c>
-      <c r="D179" s="2" t="inlineStr">
-        <is>
-          <t>Req_006, Req_015, Req_033, Req_042, Req_043, Req_045, Req_048, Req_065, Req_067, Req_068, Req_071, Req_072, Req_073, Req_074, Req_077, Req_080, Req_081, Req_087, Req_088, Req_089</t>
-        </is>
-      </c>
-      <c r="E179" s="2" t="n"/>
-      <c r="F179" s="2" t="n"/>
-      <c r="G179" s="2" t="n"/>
-      <c r="H179" s="2" t="n"/>
-    </row>
-    <row r="180">
-      <c r="A180" s="2" t="n"/>
-      <c r="B180" s="2" t="n"/>
-      <c r="C180" s="2" t="n"/>
-      <c r="D180" s="2" t="n"/>
-      <c r="E180" s="2" t="n"/>
-      <c r="F180" s="2" t="n"/>
-      <c r="G180" s="2" t="n"/>
-      <c r="H180" s="2" t="n"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="2" t="n"/>
-      <c r="B181" s="2" t="n"/>
-      <c r="C181" s="2" t="n"/>
-      <c r="D181" s="2" t="n"/>
-      <c r="E181" s="2" t="n"/>
-      <c r="F181" s="2" t="n"/>
-      <c r="G181" s="2" t="n"/>
-      <c r="H181" s="2" t="n"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="1" t="inlineStr">
-        <is>
-          <t>안전 등급 요약 (HARA 기준)</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="n"/>
-      <c r="C182" s="2" t="n"/>
-      <c r="D182" s="2" t="n"/>
-      <c r="E182" s="2" t="n"/>
-      <c r="F182" s="2" t="n"/>
-      <c r="G182" s="2" t="n"/>
-      <c r="H182" s="2" t="n"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="2" t="n"/>
-      <c r="B183" s="2" t="n"/>
-      <c r="C183" s="2" t="n"/>
-      <c r="D183" s="2" t="n"/>
-      <c r="E183" s="2" t="n"/>
-      <c r="F183" s="2" t="n"/>
-      <c r="G183" s="2" t="n"/>
-      <c r="H183" s="2" t="n"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="3" t="inlineStr">
-        <is>
-          <t>안전 등급</t>
-        </is>
-      </c>
-      <c r="B184" s="3" t="inlineStr">
-        <is>
-          <t>개수</t>
-        </is>
-      </c>
-      <c r="C184" s="3" t="inlineStr">
-        <is>
-          <t>해당 HARA ID</t>
-        </is>
-      </c>
-      <c r="D184" s="3" t="inlineStr">
-        <is>
-          <t>관련 Req (대표)</t>
-        </is>
-      </c>
-      <c r="E184" s="2" t="n"/>
-      <c r="F184" s="2" t="n"/>
-      <c r="G184" s="2" t="n"/>
-      <c r="H184" s="2" t="n"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
-        <is>
-          <t>ASIL C (Locked)</t>
-        </is>
-      </c>
-      <c r="B185" s="2" t="inlineStr">
-        <is>
-          <t>3개</t>
-        </is>
-      </c>
-      <c r="C185" s="2" t="inlineStr">
-        <is>
-          <t>HC-02, HC-03, HC-05</t>
-        </is>
-      </c>
-      <c r="D185" s="2" t="inlineStr">
-        <is>
-          <t>Req_011~Req_012, Req_021/Req_026~Req_030, Req_052~Req_056</t>
-        </is>
-      </c>
-      <c r="E185" s="2" t="n"/>
-      <c r="F185" s="2" t="n"/>
-      <c r="G185" s="2" t="n"/>
-      <c r="H185" s="2" t="n"/>
-    </row>
-    <row r="186">
-      <c r="A186" s="2" t="inlineStr">
-        <is>
-          <t>ASIL C (Provisional)</t>
-        </is>
-      </c>
-      <c r="B186" s="2" t="inlineStr">
-        <is>
-          <t>2개</t>
-        </is>
-      </c>
-      <c r="C186" s="2" t="inlineStr">
-        <is>
-          <t>HC-06, HC-07</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr">
-        <is>
-          <t>Req_057~Req_066, Req_075~Req_079</t>
-        </is>
-      </c>
-      <c r="E186" s="2" t="n"/>
-      <c r="F186" s="2" t="n"/>
-      <c r="G186" s="2" t="n"/>
-      <c r="H186" s="2" t="n"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
-        <is>
-          <t>ASIL B (Locked)</t>
-        </is>
-      </c>
-      <c r="B187" s="2" t="inlineStr">
-        <is>
-          <t>2개</t>
-        </is>
-      </c>
-      <c r="C187" s="2" t="inlineStr">
-        <is>
-          <t>HC-01, HC-04</t>
-        </is>
-      </c>
-      <c r="D187" s="2" t="inlineStr">
-        <is>
-          <t>Req_010, Req_023/Req_032/Req_033</t>
-        </is>
-      </c>
-      <c r="E187" s="2" t="n"/>
-      <c r="F187" s="2" t="n"/>
-      <c r="G187" s="2" t="n"/>
-      <c r="H187" s="2" t="n"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="2" t="inlineStr">
-        <is>
-          <t>ASIL B (Provisional)</t>
-        </is>
-      </c>
-      <c r="B188" s="2" t="inlineStr">
-        <is>
-          <t>1개</t>
-        </is>
-      </c>
-      <c r="C188" s="2" t="inlineStr">
-        <is>
-          <t>HC-08</t>
-        </is>
-      </c>
-      <c r="D188" s="2" t="inlineStr">
-        <is>
-          <t>Req_080~Req_082</t>
-        </is>
-      </c>
-      <c r="E188" s="2" t="n"/>
-      <c r="F188" s="2" t="n"/>
-      <c r="G188" s="2" t="n"/>
-      <c r="H188" s="2" t="n"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="2" t="n"/>
-      <c r="B189" s="2" t="n"/>
-      <c r="C189" s="2" t="n"/>
-      <c r="D189" s="2" t="n"/>
-      <c r="E189" s="2" t="n"/>
-      <c r="F189" s="2" t="n"/>
-      <c r="G189" s="2" t="n"/>
-      <c r="H189" s="2" t="n"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="2" t="n"/>
-      <c r="B190" s="2" t="n"/>
-      <c r="C190" s="2" t="n"/>
-      <c r="D190" s="2" t="n"/>
-      <c r="E190" s="2" t="n"/>
-      <c r="F190" s="2" t="n"/>
-      <c r="G190" s="2" t="n"/>
-      <c r="H190" s="2" t="n"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="2" t="inlineStr">
-        <is>
-          <t>안전 등급 상세 판정(원인/상황/S-E-C/안전목표)은 governance/00d_HARA_Worksheet.md를 기준으로 관리한다.</t>
-        </is>
-      </c>
-      <c r="B191" s="2" t="n"/>
-      <c r="C191" s="2" t="n"/>
-      <c r="D191" s="2" t="n"/>
-      <c r="E191" s="2" t="n"/>
-      <c r="F191" s="2" t="n"/>
-      <c r="G191" s="2" t="n"/>
-      <c r="H191" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>